<commit_message>
Updated Users test data
</commit_message>
<xml_diff>
--- a/testData/Users.xlsx
+++ b/testData/Users.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PlaywrightAutomationExercise\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7EC16EA-9DCD-43A2-BD86-C68926106659}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D1A5F40-5A54-4F25-82AA-50FA79B16DC8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="12010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -87,9 +87,6 @@
     <t>456 New Street</t>
   </si>
   <si>
-    <t>Awan Town</t>
-  </si>
-  <si>
     <t>United States</t>
   </si>
   <si>
@@ -126,9 +123,6 @@
     <t>123 Test Street</t>
   </si>
   <si>
-    <t>Multan Road</t>
-  </si>
-  <si>
     <t>static</t>
   </si>
   <si>
@@ -268,6 +262,12 @@
   </si>
   <si>
     <t>90002</t>
+  </si>
+  <si>
+    <t>Los Angeles Street 1</t>
+  </si>
+  <si>
+    <t>Los Angeles Street 2</t>
   </si>
 </sst>
 </file>
@@ -544,7 +544,7 @@
     <col min="5" max="5" width="9.4140625" customWidth="1"/>
     <col min="6" max="6" width="19.08203125" customWidth="1"/>
     <col min="7" max="7" width="13.75" customWidth="1"/>
-    <col min="8" max="8" width="8.08203125" customWidth="1"/>
+    <col min="8" max="8" width="19" customWidth="1"/>
     <col min="9" max="9" width="11.75" customWidth="1"/>
     <col min="10" max="10" width="8.83203125" customWidth="1"/>
     <col min="11" max="11" width="10.25" customWidth="1"/>
@@ -620,69 +620,69 @@
         <v>20</v>
       </c>
       <c r="H2" t="s">
+        <v>80</v>
+      </c>
+      <c r="I2" t="s">
         <v>21</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>22</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>23</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>24</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>25</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>26</v>
-      </c>
-      <c r="N2" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>29</v>
       </c>
       <c r="C3" t="s">
         <v>16</v>
       </c>
       <c r="D3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" t="s">
         <v>30</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>31</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>32</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
+        <v>81</v>
+      </c>
+      <c r="I3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K3" t="s">
+        <v>23</v>
+      </c>
+      <c r="L3" t="s">
+        <v>79</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="N3" t="s">
         <v>33</v>
-      </c>
-      <c r="H3" t="s">
-        <v>34</v>
-      </c>
-      <c r="I3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J3" t="s">
-        <v>23</v>
-      </c>
-      <c r="K3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L3" t="s">
-        <v>81</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="N3" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -712,7 +712,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
         <v>15</v>
@@ -723,13 +723,13 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" t="s">
         <v>37</v>
-      </c>
-      <c r="B3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C3" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -747,162 +747,162 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B12" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B13" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B17" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B18" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B19" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B20" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>